<commit_message>
Fase 5: módulo Vencimientos (Previsión + cargos repetidos detectados)
- A: tblProgramados con la nueva columna «Día», por frecuencia, desde/hasta y cruzando de año
- B: cargos de ≥3 meses, mensual o trimestral (±5 días), importe ±15 %, recibos del mismo día sumados
- Próximos 30 días, aviso a 7 días, solo tu parte; descarta duplicados con Previsión y cargos ajenos
- Mismo desbloqueo y lectura del Excel que Finanzas; no se carga en el PC de trabajo
- Tests con un libro sintético; comprobado con el Excel real

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013YdsV3oVQn7fHoHAaRE9EA
</commit_message>
<xml_diff>
--- a/src/lib/fixtures/cuentas-prueba.xlsx
+++ b/src/lib/fixtures/cuentas-prueba.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importar" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movimientos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorías" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Previsión" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorías" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="cfgAnio">Importar!$C$23</definedName>
@@ -153,6 +154,24 @@
     <tableColumn id="5" name="Importe"/>
     <tableColumn id="6" name="Categoría"/>
     <tableColumn id="7" name="Corresponde Germán"/>
+  </tableColumns>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblProgramados" displayName="tblProgramados" ref="A1:J6" headerRowCount="1">
+  <autoFilter ref="A1:J6"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Concepto"/>
+    <tableColumn id="2" name="Categoría"/>
+    <tableColumn id="3" name="Importe"/>
+    <tableColumn id="4" name="Tipo de gasto"/>
+    <tableColumn id="5" name="Frecuencia"/>
+    <tableColumn id="6" name="Desde"/>
+    <tableColumn id="7" name="Hasta"/>
+    <tableColumn id="8" name="Estado"/>
+    <tableColumn id="9" name="% Germán"/>
+    <tableColumn id="10" name="Día"/>
   </tableColumns>
 </table>
 </file>
@@ -972,6 +991,279 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Importe</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Tipo de gasto</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Frecuencia</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Desde</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Hasta</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>% Germán</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Seguro hogar</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>240</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Compartido</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cuota comunidad</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Comunidad</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>264.21</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Compartido</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Trimestral</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>IBI</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>290.41</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Compartido</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Derrama</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Comunidad</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Compartido</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gimnasio programado</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Deporte/Panteres</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Individual Germán</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>